<commit_message>
docs(order-history): record SBE-1147 nesting + SBE-1146 invoice rework on the 13.3 docs
Both merged to dev and previously undocumented. GET /orders/:orderId is
now product-gated and nested-by-show (shows[] with per-show booths/add_ons/
sponsorships/onsite_contact, unassigned bucket, product_name/purchased_name,
per-booth setup_fee/cleaning_fee, additional_purchases[].show); the invoice
route was split into GET /orders/:orderId/invoices (list) + GET /orders/
invoices/:id (download by id), replacing the old latest-only route.

Updated 13.3 feasibility .md/.xlsx, orders-guide capability + contract
(md/mmd/regenerated svg) + endpoint catalog, feasibility summary xlsx, and
the build consolidation reuse map; added the SBE-1147 implementation plan.
</commit_message>
<xml_diff>
--- a/order_history/_Order History - Feasibility Summary.xlsx
+++ b/order_history/_Order History - Feasibility Summary.xlsx
@@ -714,11 +714,11 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>25 to build</t>
+          <t>25 to build (+ post-ship reworks SBE-1146 invoice endpoints 2026-07-17 &amp; SBE-1147 nesting 2026-07-26)</t>
         </is>
       </c>
       <c r="K4" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L4" s="2" t="n">
         <v>3</v>
@@ -773,7 +773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -861,7 +861,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Read-only Order Details aggregate: header, booth/add-on/sponsorship line items, financial summary, payment details + schedule, agreement acceptance. Ownership-scoped to the requesting exhibitor's company.</t>
+          <t>Read-only Order Details aggregate — NESTED BY SHOW (SBE-1147, 2026-07-26): shows[] each with its booths/add_ons/sponsorships + onsite_contact, plus financial_summary, settled payments[], agreement, additional_purchases[].show, nullable 'unassigned' bucket, can_download_invoice. PRODUCT-GATED (subscription/ppl_addon -&gt; 404).</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -876,7 +876,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Navigated from a row in the GET /orders listing. The 13.2 'View action opens the detailed order summary' requirement (13.2-f) reuses this endpoint — no separate route in 13.2.</t>
+          <t>Navigated from a row in the GET /orders listing. The 13.2 'View action opens the detailed order summary' requirement (13.2-f) reuses this endpoint — no separate route in 13.2. | SBE-1147 (2026-07-26, PR #372) restructured the response nested-by-show + product-gated; DTO is OrderDetailShowDto (distinct from the 13.2-shared OrderShowDto).</t>
         </is>
       </c>
     </row>
@@ -888,12 +888,12 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>/orders/:orderId/invoice</t>
+          <t>/orders/invoices/:id</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Generate/return the invoice PDF (pdfkit render + signed URL), reusing the existing PPL downloadInvoicePdf/renderInvoicePdf path; split orders may expose per-installment invoices.</t>
+          <t>Download a SPECIFIC invoice PDF by invoice id (pdfkit render + signed URL), Option B / product-gated / paid-only. Replaced the old latest-only /orders/:orderId/invoice (invoice rework SBE-1146, 2026-07-17).</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -908,7 +908,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Shared by the 13.2 listing Invoice action and the 13.3 details-page Download Invoice button — one endpoint, not two.</t>
+          <t>Shared by the 13.2 listing Invoice action and the 13.3 details-page Download Invoice button — one endpoint, not two. | SBE-1146 rework: per-invoice download by id (was latest-only); ids come from GET /orders/:orderId/invoices.</t>
         </is>
       </c>
     </row>
@@ -920,25 +920,57 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
+          <t>/orders/:orderId/invoices</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>List every invoice on one product order (newest first: id, invoice_number, status, total, paid_at, created_at); 200 empty list when none yet. Feeds ids to GET /orders/invoices/:id.</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>13.3</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>13.3-s</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>NEW in the invoice rework (SBE-1146, 2026-07-17) — makes split orders' older invoices reachable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
           <t>/orders/:orderId/agreement</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Download the stored signed agreement (PDF / signature record + acceptance metadata) for the order.</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>13.3</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>13.3-v, 13.3-ac</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Distinct document from the invoice — NOT merged with /orders/:orderId/invoice. Only 13.3 uses it.</t>
         </is>

</xml_diff>